<commit_message>
Changed dead timing and ran optimization again. Generated new excel list
</commit_message>
<xml_diff>
--- a/Mosfet_extraction_pipeline/excel_sheets/low_side_frequency_matrix_LM5106.xlsx
+++ b/Mosfet_extraction_pipeline/excel_sheets/low_side_frequency_matrix_LM5106.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sync_Buck_convertor\Mosfet_extraction_pipeline\excel_sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7318F1DE-CA4B-4A40-941E-05788B455A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B29DC3-3E1F-458F-9F97-51760359B176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="17">
   <si>
     <t>Frequency_kHz</t>
   </si>
@@ -52,22 +52,13 @@
     <t>Ratio</t>
   </si>
   <si>
+    <t>Infineon BSC014N04LSI</t>
+  </si>
+  <si>
     <t>Infineon IAUAN04S7N005</t>
   </si>
   <si>
     <t>Infineon IAUAN04S7N006</t>
-  </si>
-  <si>
-    <t>Infineon IQDH45N04LM6CGSC</t>
-  </si>
-  <si>
-    <t>Infineon IQD005N04NM6SC</t>
-  </si>
-  <si>
-    <t>Infineon IAUCN04S7N006T</t>
-  </si>
-  <si>
-    <t>Infineon BSC014N04LSI</t>
   </si>
   <si>
     <t>Infineon IAUTN06S5N008G</t>
@@ -77,6 +68,9 @@
   </si>
   <si>
     <t>Comchip Technology CMS23N06H8-HF</t>
+  </si>
+  <si>
+    <t>Analog Power AM4362N</t>
   </si>
 </sst>
 </file>
@@ -426,9 +420,8 @@
   <dimension ref="A1:J146"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="39.54296875" customWidth="1"/>
-    <col min="4" max="4" width="16.36328125" customWidth="1"/>
-    <col min="5" max="5" width="13.7265625" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="28.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -474,25 +467,25 @@
         <v>10</v>
       </c>
       <c r="D2">
-        <v>5.7426164772727273E-2</v>
+        <v>9.822144886363636E-2</v>
       </c>
       <c r="E2">
-        <v>0.11</v>
+        <v>5.5E-2</v>
       </c>
       <c r="F2">
-        <v>0.51</v>
+        <v>1.45</v>
       </c>
       <c r="G2">
-        <v>37.5</v>
+        <v>12</v>
       </c>
       <c r="H2">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="I2">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="J2">
-        <v>2.9333333333333331</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -506,25 +499,25 @@
         <v>11</v>
       </c>
       <c r="D3">
-        <v>5.8593948863636357E-2</v>
+        <v>0.1049261647727273</v>
       </c>
       <c r="E3">
-        <v>9.4000000000000014E-2</v>
+        <v>0.11</v>
       </c>
       <c r="F3">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G3">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H3">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I3">
         <v>0.95</v>
       </c>
       <c r="J3">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -538,25 +531,25 @@
         <v>12</v>
       </c>
       <c r="D4">
-        <v>5.9536903409090902E-2</v>
+        <v>0.10609394886363641</v>
       </c>
       <c r="E4">
-        <v>0.129</v>
+        <v>9.4000000000000014E-2</v>
       </c>
       <c r="F4">
-        <v>0.49</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G4">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H4">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="J4">
-        <v>5.6086956521739131</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -570,25 +563,25 @@
         <v>13</v>
       </c>
       <c r="D5">
-        <v>5.9536903409090902E-2</v>
+        <v>0.10718119318181819</v>
       </c>
       <c r="E5">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="F5">
-        <v>0.49</v>
+        <v>0.78</v>
       </c>
       <c r="G5">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="H5">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="J5">
-        <v>4.8099999999999996</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -602,25 +595,25 @@
         <v>14</v>
       </c>
       <c r="D6">
-        <v>5.9956363636363641E-2</v>
+        <v>0.10737582386363639</v>
       </c>
       <c r="E6">
-        <v>0.112</v>
+        <v>0.21</v>
       </c>
       <c r="F6">
-        <v>0.64</v>
+        <v>0.79</v>
       </c>
       <c r="G6">
-        <v>39.5</v>
+        <v>68</v>
       </c>
       <c r="H6">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="I6">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J6">
-        <v>2.835443037974684</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -634,25 +627,25 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>6.9301164772727269E-2</v>
+        <v>0.1157214488636364</v>
       </c>
       <c r="E7">
-        <v>0.13750000000000001</v>
+        <v>6.8750000000000006E-2</v>
       </c>
       <c r="F7">
-        <v>0.51</v>
+        <v>1.45</v>
       </c>
       <c r="G7">
-        <v>37.5</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="I7">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
       <c r="J7">
-        <v>2.9333333333333331</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -666,25 +659,25 @@
         <v>11</v>
       </c>
       <c r="D8">
-        <v>7.046894886363636E-2</v>
+        <v>0.12867616477272731</v>
       </c>
       <c r="E8">
-        <v>0.11749999999999999</v>
+        <v>0.13750000000000001</v>
       </c>
       <c r="F8">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G8">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H8">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I8">
         <v>0.95</v>
       </c>
       <c r="J8">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -695,28 +688,28 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>7.1831363636363638E-2</v>
+        <v>0.1298439488636364</v>
       </c>
       <c r="E9">
-        <v>0.14000000000000001</v>
+        <v>0.11749999999999999</v>
       </c>
       <c r="F9">
-        <v>0.64</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G9">
-        <v>39.5</v>
+        <v>32</v>
       </c>
       <c r="H9">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="I9">
         <v>0.95</v>
       </c>
       <c r="J9">
-        <v>2.835443037974684</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -727,28 +720,28 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10">
-        <v>7.1971448863636364E-2</v>
+        <v>0.1301811931818182</v>
       </c>
       <c r="E10">
-        <v>6.8750000000000006E-2</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="F10">
-        <v>1.45</v>
+        <v>0.78</v>
       </c>
       <c r="G10">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="H10">
-        <v>55</v>
+        <v>210</v>
       </c>
       <c r="I10">
-        <v>0.7</v>
+        <v>0.92</v>
       </c>
       <c r="J10">
-        <v>4.58</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -759,28 +752,28 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D11">
-        <v>7.2036903409090913E-2</v>
+        <v>0.13037582386363639</v>
       </c>
       <c r="E11">
-        <v>0.16125</v>
+        <v>0.26250000000000001</v>
       </c>
       <c r="F11">
-        <v>0.49</v>
+        <v>0.79</v>
       </c>
       <c r="G11">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="H11">
-        <v>129</v>
+        <v>210</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="J11">
-        <v>5.6086956521739131</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -791,10 +784,10 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D12">
-        <v>8.0721448863636358E-2</v>
+        <v>0.13322144886363629</v>
       </c>
       <c r="E12">
         <v>8.2500000000000004E-2</v>
@@ -823,10 +816,10 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D13">
-        <v>8.1176164772727266E-2</v>
+        <v>0.15242616477272719</v>
       </c>
       <c r="E13">
         <v>0.16500000000000001</v>
@@ -855,28 +848,28 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14">
-        <v>8.2343948863636357E-2</v>
+        <v>0.15318119318181819</v>
       </c>
       <c r="E14">
-        <v>0.14099999999999999</v>
+        <v>0.31500000000000011</v>
       </c>
       <c r="F14">
-        <v>0.56999999999999995</v>
+        <v>0.78</v>
       </c>
       <c r="G14">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="H14">
-        <v>94</v>
+        <v>210</v>
       </c>
       <c r="I14">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J14">
-        <v>2.9375</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -890,25 +883,25 @@
         <v>14</v>
       </c>
       <c r="D15">
-        <v>8.3706363636363634E-2</v>
+        <v>0.15337582386363641</v>
       </c>
       <c r="E15">
-        <v>0.16800000000000001</v>
+        <v>0.31500000000000011</v>
       </c>
       <c r="F15">
-        <v>0.64</v>
+        <v>0.79</v>
       </c>
       <c r="G15">
-        <v>39.5</v>
+        <v>68</v>
       </c>
       <c r="H15">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="I15">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J15">
-        <v>2.835443037974684</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -919,28 +912,28 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D16">
-        <v>8.4181193181818187E-2</v>
+        <v>0.15359394886363639</v>
       </c>
       <c r="E16">
-        <v>0.31500000000000011</v>
+        <v>0.14099999999999999</v>
       </c>
       <c r="F16">
-        <v>0.78</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G16">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H16">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I16">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J16">
-        <v>3.0882350000000001</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -951,10 +944,10 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D17">
-        <v>8.9471448863636366E-2</v>
+        <v>0.15072144886363639</v>
       </c>
       <c r="E17">
         <v>9.6250000000000002E-2</v>
@@ -983,10 +976,10 @@
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D18">
-        <v>9.3051164772727277E-2</v>
+        <v>0.1761761647727273</v>
       </c>
       <c r="E18">
         <v>0.1925</v>
@@ -1015,28 +1008,28 @@
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D19">
-        <v>9.4218948863636368E-2</v>
+        <v>0.17618119318181821</v>
       </c>
       <c r="E19">
-        <v>0.16450000000000001</v>
+        <v>0.36749999999999999</v>
       </c>
       <c r="F19">
-        <v>0.56999999999999995</v>
+        <v>0.78</v>
       </c>
       <c r="G19">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="H19">
-        <v>94</v>
+        <v>210</v>
       </c>
       <c r="I19">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J19">
-        <v>2.9375</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1050,25 +1043,25 @@
         <v>14</v>
       </c>
       <c r="D20">
-        <v>9.5581363636363645E-2</v>
+        <v>0.1763758238636364</v>
       </c>
       <c r="E20">
-        <v>0.19600000000000001</v>
+        <v>0.36749999999999999</v>
       </c>
       <c r="F20">
-        <v>0.64</v>
+        <v>0.79</v>
       </c>
       <c r="G20">
-        <v>39.5</v>
+        <v>68</v>
       </c>
       <c r="H20">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="I20">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J20">
-        <v>2.835443037974684</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -1079,28 +1072,28 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D21">
-        <v>9.5681193181818183E-2</v>
+        <v>0.17734394886363641</v>
       </c>
       <c r="E21">
-        <v>0.36749999999999999</v>
+        <v>0.16450000000000001</v>
       </c>
       <c r="F21">
-        <v>0.78</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G21">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H21">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I21">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J21">
-        <v>3.0882350000000001</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -1111,10 +1104,10 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D22">
-        <v>9.822144886363636E-2</v>
+        <v>0.16822144886363641</v>
       </c>
       <c r="E22">
         <v>0.11</v>
@@ -1143,28 +1136,28 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D23">
-        <v>0.1049261647727273</v>
+        <v>0.19918119318181821</v>
       </c>
       <c r="E23">
-        <v>0.22</v>
+        <v>0.42</v>
       </c>
       <c r="F23">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G23">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H23">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I23">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J23">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -1175,28 +1168,28 @@
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D24">
-        <v>0.10609394886363641</v>
+        <v>0.19937582386363639</v>
       </c>
       <c r="E24">
-        <v>0.188</v>
+        <v>0.42</v>
       </c>
       <c r="F24">
-        <v>0.56999999999999995</v>
+        <v>0.79</v>
       </c>
       <c r="G24">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="H24">
-        <v>94</v>
+        <v>210</v>
       </c>
       <c r="I24">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J24">
-        <v>2.9375</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -1207,28 +1200,28 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D25">
-        <v>0.10718119318181819</v>
+        <v>0.19992616477272729</v>
       </c>
       <c r="E25">
-        <v>0.42</v>
+        <v>0.22</v>
       </c>
       <c r="F25">
-        <v>0.78</v>
+        <v>0.51</v>
       </c>
       <c r="G25">
-        <v>68</v>
+        <v>37.5</v>
       </c>
       <c r="H25">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="I25">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J25">
-        <v>3.0882350000000001</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -1239,28 +1232,28 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D26">
-        <v>0.10737582386363639</v>
+        <v>0.20109394886363641</v>
       </c>
       <c r="E26">
-        <v>0.42</v>
+        <v>0.188</v>
       </c>
       <c r="F26">
-        <v>0.79</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G26">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H26">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I26">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J26">
-        <v>3.0882352941176472</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -1271,10 +1264,10 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D27">
-        <v>0.1069714488636364</v>
+        <v>0.1857214488636364</v>
       </c>
       <c r="E27">
         <v>0.12375</v>
@@ -1303,28 +1296,28 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D28">
-        <v>0.1168011647727273</v>
+        <v>0.2221811931818182</v>
       </c>
       <c r="E28">
-        <v>0.2475</v>
+        <v>0.47249999999999998</v>
       </c>
       <c r="F28">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G28">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H28">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I28">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J28">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
@@ -1335,28 +1328,28 @@
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D29">
-        <v>0.1179689488636364</v>
+        <v>0.22237582386363641</v>
       </c>
       <c r="E29">
-        <v>0.21149999999999999</v>
+        <v>0.47249999999999998</v>
       </c>
       <c r="F29">
-        <v>0.56999999999999995</v>
+        <v>0.79</v>
       </c>
       <c r="G29">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="H29">
-        <v>94</v>
+        <v>210</v>
       </c>
       <c r="I29">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J29">
-        <v>2.9375</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -1367,28 +1360,28 @@
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D30">
-        <v>0.1186811931818182</v>
+        <v>0.22367616477272731</v>
       </c>
       <c r="E30">
-        <v>0.47249999999999998</v>
+        <v>0.2475</v>
       </c>
       <c r="F30">
-        <v>0.78</v>
+        <v>0.51</v>
       </c>
       <c r="G30">
-        <v>68</v>
+        <v>37.5</v>
       </c>
       <c r="H30">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="I30">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J30">
-        <v>3.0882350000000001</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
@@ -1399,28 +1392,28 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D31">
-        <v>0.1188758238636364</v>
+        <v>0.22484394886363629</v>
       </c>
       <c r="E31">
-        <v>0.47249999999999998</v>
+        <v>0.21149999999999999</v>
       </c>
       <c r="F31">
-        <v>0.79</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G31">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H31">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I31">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J31">
-        <v>3.0882352941176472</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -1431,10 +1424,10 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D32">
-        <v>0.1157214488636364</v>
+        <v>0.20322144886363641</v>
       </c>
       <c r="E32">
         <v>0.13750000000000001</v>
@@ -1463,28 +1456,28 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D33">
-        <v>0.12867616477272731</v>
+        <v>0.24518119318181819</v>
       </c>
       <c r="E33">
-        <v>0.27500000000000002</v>
+        <v>0.52500000000000002</v>
       </c>
       <c r="F33">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G33">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H33">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I33">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J33">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
@@ -1495,28 +1488,28 @@
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D34">
-        <v>0.1298439488636364</v>
+        <v>0.24537582386363641</v>
       </c>
       <c r="E34">
-        <v>0.23499999999999999</v>
+        <v>0.52500000000000002</v>
       </c>
       <c r="F34">
-        <v>0.56999999999999995</v>
+        <v>0.79</v>
       </c>
       <c r="G34">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="H34">
-        <v>94</v>
+        <v>210</v>
       </c>
       <c r="I34">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J34">
-        <v>2.9375</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
@@ -1527,28 +1520,28 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D35">
-        <v>0.1301811931818182</v>
+        <v>0.2474261647727273</v>
       </c>
       <c r="E35">
-        <v>0.52500000000000002</v>
+        <v>0.27500000000000002</v>
       </c>
       <c r="F35">
-        <v>0.78</v>
+        <v>0.51</v>
       </c>
       <c r="G35">
-        <v>68</v>
+        <v>37.5</v>
       </c>
       <c r="H35">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="I35">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J35">
-        <v>3.0882350000000001</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
@@ -1559,28 +1552,28 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D36">
-        <v>0.13037582386363639</v>
+        <v>0.24859394886363631</v>
       </c>
       <c r="E36">
-        <v>0.52500000000000002</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="F36">
-        <v>0.79</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G36">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H36">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I36">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J36">
-        <v>3.0882352941176472</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
@@ -1591,10 +1584,10 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D37">
-        <v>0.1244714488636364</v>
+        <v>0.2207214488636364</v>
       </c>
       <c r="E37">
         <v>0.15125</v>
@@ -1623,28 +1616,28 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D38">
-        <v>0.14055116477272731</v>
+        <v>0.26818119318181821</v>
       </c>
       <c r="E38">
-        <v>0.30249999999999999</v>
+        <v>0.57750000000000001</v>
       </c>
       <c r="F38">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G38">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H38">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I38">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J38">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
@@ -1655,16 +1648,16 @@
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D39">
-        <v>0.14168119318181821</v>
+        <v>0.26837582386363629</v>
       </c>
       <c r="E39">
         <v>0.57750000000000001</v>
       </c>
       <c r="F39">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="G39">
         <v>68</v>
@@ -1676,7 +1669,7 @@
         <v>0.92</v>
       </c>
       <c r="J39">
-        <v>3.0882350000000001</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
@@ -1690,25 +1683,25 @@
         <v>11</v>
       </c>
       <c r="D40">
-        <v>0.14171894886363631</v>
+        <v>0.27117616477272732</v>
       </c>
       <c r="E40">
-        <v>0.25850000000000001</v>
+        <v>0.30249999999999999</v>
       </c>
       <c r="F40">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G40">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H40">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I40">
         <v>0.95</v>
       </c>
       <c r="J40">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
@@ -1719,28 +1712,28 @@
         <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D41">
-        <v>0.1418758238636364</v>
+        <v>0.27234394886363628</v>
       </c>
       <c r="E41">
-        <v>0.57750000000000001</v>
+        <v>0.25850000000000001</v>
       </c>
       <c r="F41">
-        <v>0.79</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="G41">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="H41">
-        <v>210</v>
+        <v>94</v>
       </c>
       <c r="I41">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J41">
-        <v>3.0882352941176472</v>
+        <v>2.9375</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
@@ -1751,10 +1744,10 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D42">
-        <v>0.13322144886363629</v>
+        <v>0.23822144886363639</v>
       </c>
       <c r="E42">
         <v>0.16500000000000001</v>
@@ -1783,28 +1776,28 @@
         <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D43">
-        <v>0.15242616477272719</v>
+        <v>0.29118119318181818</v>
       </c>
       <c r="E43">
-        <v>0.33</v>
+        <v>0.63000000000000012</v>
       </c>
       <c r="F43">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G43">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H43">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I43">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J43">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
@@ -1815,16 +1808,16 @@
         <v>3</v>
       </c>
       <c r="C44" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D44">
-        <v>0.15318119318181819</v>
+        <v>0.29137582386363642</v>
       </c>
       <c r="E44">
         <v>0.63000000000000012</v>
       </c>
       <c r="F44">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="G44">
         <v>68</v>
@@ -1836,7 +1829,7 @@
         <v>0.92</v>
       </c>
       <c r="J44">
-        <v>3.0882350000000001</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
@@ -1847,28 +1840,28 @@
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D45">
-        <v>0.15337582386363641</v>
+        <v>0.29492616477272732</v>
       </c>
       <c r="E45">
-        <v>0.63000000000000012</v>
+        <v>0.33</v>
       </c>
       <c r="F45">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
       <c r="G45">
-        <v>68</v>
+        <v>37.5</v>
       </c>
       <c r="H45">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="I45">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J45">
-        <v>3.0882352941176472</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
@@ -1879,10 +1872,10 @@
         <v>5</v>
       </c>
       <c r="C46" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D46">
-        <v>0.15359394886363639</v>
+        <v>0.29609394886363632</v>
       </c>
       <c r="E46">
         <v>0.28199999999999997</v>
@@ -1911,10 +1904,10 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D47">
-        <v>0.14197144886363641</v>
+        <v>0.25572144886363629</v>
       </c>
       <c r="E47">
         <v>0.17874999999999999</v>
@@ -1943,28 +1936,28 @@
         <v>2</v>
       </c>
       <c r="C48" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D48">
-        <v>0.1643011647727273</v>
+        <v>0.31418119318181831</v>
       </c>
       <c r="E48">
-        <v>0.35749999999999998</v>
+        <v>0.68250000000000011</v>
       </c>
       <c r="F48">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G48">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H48">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I48">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J48">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
@@ -1975,16 +1968,16 @@
         <v>3</v>
       </c>
       <c r="C49" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D49">
-        <v>0.1646811931818182</v>
+        <v>0.31437582386363638</v>
       </c>
       <c r="E49">
         <v>0.68250000000000011</v>
       </c>
       <c r="F49">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="G49">
         <v>68</v>
@@ -1996,7 +1989,7 @@
         <v>0.92</v>
       </c>
       <c r="J49">
-        <v>3.0882350000000001</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
@@ -2007,28 +2000,28 @@
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D50">
-        <v>0.16487582386363639</v>
+        <v>0.31867616477272731</v>
       </c>
       <c r="E50">
-        <v>0.68250000000000011</v>
+        <v>0.35749999999999998</v>
       </c>
       <c r="F50">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
       <c r="G50">
-        <v>68</v>
+        <v>37.5</v>
       </c>
       <c r="H50">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="I50">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="J50">
-        <v>3.0882352941176472</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
@@ -2039,10 +2032,10 @@
         <v>5</v>
       </c>
       <c r="C51" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D51">
-        <v>0.16546894886363639</v>
+        <v>0.31984394886363637</v>
       </c>
       <c r="E51">
         <v>0.30549999999999999</v>
@@ -2071,10 +2064,10 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D52">
-        <v>0.15072144886363639</v>
+        <v>0.27322144886363642</v>
       </c>
       <c r="E52">
         <v>0.1925</v>
@@ -2103,28 +2096,28 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D53">
-        <v>0.1761761647727273</v>
+        <v>0.33718119318181822</v>
       </c>
       <c r="E53">
-        <v>0.38500000000000001</v>
+        <v>0.7350000000000001</v>
       </c>
       <c r="F53">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="G53">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H53">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I53">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J53">
-        <v>2.9333333333333331</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
@@ -2135,16 +2128,16 @@
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D54">
-        <v>0.17618119318181821</v>
+        <v>0.33737582386363629</v>
       </c>
       <c r="E54">
         <v>0.7350000000000001</v>
       </c>
       <c r="F54">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="G54">
         <v>68</v>
@@ -2156,7 +2149,7 @@
         <v>0.92</v>
       </c>
       <c r="J54">
-        <v>3.0882350000000001</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
@@ -2167,28 +2160,28 @@
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D55">
-        <v>0.1763758238636364</v>
+        <v>0.34033551136363632</v>
       </c>
       <c r="E55">
-        <v>0.7350000000000001</v>
+        <v>0.224</v>
       </c>
       <c r="F55">
-        <v>0.79</v>
+        <v>3.1</v>
       </c>
       <c r="G55">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="H55">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I55">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J55">
-        <v>3.0882352941176472</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
@@ -2202,25 +2195,25 @@
         <v>11</v>
       </c>
       <c r="D56">
-        <v>0.17734394886363641</v>
+        <v>0.3424261647727273</v>
       </c>
       <c r="E56">
-        <v>0.32900000000000001</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="F56">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G56">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H56">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I56">
         <v>0.95</v>
       </c>
       <c r="J56">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
@@ -2231,10 +2224,10 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D57">
-        <v>0.1594714488636364</v>
+        <v>0.29072144886363638</v>
       </c>
       <c r="E57">
         <v>0.20624999999999999</v>
@@ -2263,10 +2256,10 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D58">
-        <v>0.1876811931818182</v>
+        <v>0.36018119318181818</v>
       </c>
       <c r="E58">
         <v>0.78750000000000009</v>
@@ -2295,28 +2288,28 @@
         <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D59">
-        <v>0.18787582386363641</v>
+        <v>0.36033551136363628</v>
       </c>
       <c r="E59">
-        <v>0.78750000000000009</v>
+        <v>0.24</v>
       </c>
       <c r="F59">
-        <v>0.79</v>
+        <v>3.1</v>
       </c>
       <c r="G59">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="H59">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I59">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J59">
-        <v>3.0882352941176472</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
@@ -2327,28 +2320,28 @@
         <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D60">
-        <v>0.18805116477272729</v>
+        <v>0.36037582386363642</v>
       </c>
       <c r="E60">
-        <v>0.41249999999999998</v>
+        <v>0.78750000000000009</v>
       </c>
       <c r="F60">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G60">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H60">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I60">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J60">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
@@ -2362,25 +2355,25 @@
         <v>11</v>
       </c>
       <c r="D61">
-        <v>0.18921894886363641</v>
+        <v>0.3661761647727273</v>
       </c>
       <c r="E61">
-        <v>0.35249999999999998</v>
+        <v>0.41249999999999998</v>
       </c>
       <c r="F61">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G61">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H61">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I61">
         <v>0.95</v>
       </c>
       <c r="J61">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
@@ -2391,10 +2384,10 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D62">
-        <v>0.16822144886363641</v>
+        <v>0.30822144886363628</v>
       </c>
       <c r="E62">
         <v>0.22</v>
@@ -2423,28 +2416,28 @@
         <v>2</v>
       </c>
       <c r="C63" t="s">
+        <v>15</v>
+      </c>
+      <c r="D63">
+        <v>0.38033551136363641</v>
+      </c>
+      <c r="E63">
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="F63">
+        <v>3.1</v>
+      </c>
+      <c r="G63">
         <v>16</v>
       </c>
-      <c r="D63">
-        <v>0.19918119318181821</v>
-      </c>
-      <c r="E63">
-        <v>0.84000000000000008</v>
-      </c>
-      <c r="F63">
-        <v>0.78</v>
-      </c>
-      <c r="G63">
-        <v>68</v>
-      </c>
       <c r="H63">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I63">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J63">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
@@ -2455,16 +2448,16 @@
         <v>3</v>
       </c>
       <c r="C64" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D64">
-        <v>0.19937582386363639</v>
+        <v>0.38318119318181831</v>
       </c>
       <c r="E64">
         <v>0.84000000000000008</v>
       </c>
       <c r="F64">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G64">
         <v>68</v>
@@ -2476,7 +2469,7 @@
         <v>0.92</v>
       </c>
       <c r="J64">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
@@ -2487,28 +2480,28 @@
         <v>4</v>
       </c>
       <c r="C65" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D65">
-        <v>0.19992616477272729</v>
+        <v>0.38337582386363639</v>
       </c>
       <c r="E65">
-        <v>0.44</v>
+        <v>0.84000000000000008</v>
       </c>
       <c r="F65">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G65">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H65">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I65">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J65">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
@@ -2522,56 +2515,56 @@
         <v>11</v>
       </c>
       <c r="D66">
-        <v>0.20109394886363641</v>
+        <v>0.38992616477272729</v>
       </c>
       <c r="E66">
-        <v>0.37600000000000011</v>
+        <v>0.44</v>
       </c>
       <c r="F66">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G66">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H66">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I66">
         <v>0.95</v>
       </c>
       <c r="J66">
-        <v>2.9375</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67">
+        <v>2.9333333333333331</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
         <v>425</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="1">
         <v>1</v>
       </c>
-      <c r="C67" t="s">
-        <v>15</v>
-      </c>
-      <c r="D67">
-        <v>0.17697144886363639</v>
-      </c>
-      <c r="E67">
+      <c r="C67" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D67" s="1">
+        <v>0.32572144886363641</v>
+      </c>
+      <c r="E67" s="1">
         <v>0.23375000000000001</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="1">
         <v>1.45</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="1">
         <v>12</v>
       </c>
-      <c r="H67">
+      <c r="H67" s="1">
         <v>55</v>
       </c>
-      <c r="I67">
+      <c r="I67" s="1">
         <v>0.7</v>
       </c>
-      <c r="J67">
+      <c r="J67" s="1">
         <v>4.58</v>
       </c>
     </row>
@@ -2583,28 +2576,28 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
+        <v>15</v>
+      </c>
+      <c r="D68">
+        <v>0.40033551136363632</v>
+      </c>
+      <c r="E68">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="F68">
+        <v>3.1</v>
+      </c>
+      <c r="G68">
         <v>16</v>
       </c>
-      <c r="D68">
-        <v>0.21068119318181819</v>
-      </c>
-      <c r="E68">
-        <v>0.89250000000000007</v>
-      </c>
-      <c r="F68">
-        <v>0.78</v>
-      </c>
-      <c r="G68">
-        <v>68</v>
-      </c>
       <c r="H68">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I68">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J68">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
@@ -2615,16 +2608,16 @@
         <v>3</v>
       </c>
       <c r="C69" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D69">
-        <v>0.2108758238636364</v>
+        <v>0.40618119318181822</v>
       </c>
       <c r="E69">
         <v>0.89250000000000007</v>
       </c>
       <c r="F69">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G69">
         <v>68</v>
@@ -2636,7 +2629,7 @@
         <v>0.92</v>
       </c>
       <c r="J69">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
@@ -2647,28 +2640,28 @@
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D70">
-        <v>0.21180116477272731</v>
+        <v>0.40637582386363641</v>
       </c>
       <c r="E70">
-        <v>0.46750000000000003</v>
+        <v>0.89250000000000007</v>
       </c>
       <c r="F70">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G70">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H70">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I70">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J70">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
@@ -2682,56 +2675,56 @@
         <v>11</v>
       </c>
       <c r="D71">
-        <v>0.2129689488636364</v>
+        <v>0.41367616477272728</v>
       </c>
       <c r="E71">
-        <v>0.39950000000000002</v>
+        <v>0.46750000000000003</v>
       </c>
       <c r="F71">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G71">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H71">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I71">
         <v>0.95</v>
       </c>
       <c r="J71">
-        <v>2.9375</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="1">
+        <v>2.9333333333333331</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A72">
         <v>450</v>
       </c>
-      <c r="B72" s="1">
+      <c r="B72">
         <v>1</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D72" s="1">
-        <v>0.1857214488636364</v>
-      </c>
-      <c r="E72" s="1">
+      <c r="C72" t="s">
+        <v>10</v>
+      </c>
+      <c r="D72">
+        <v>0.34322144886363642</v>
+      </c>
+      <c r="E72">
         <v>0.2475</v>
       </c>
-      <c r="F72" s="1">
+      <c r="F72">
         <v>1.45</v>
       </c>
-      <c r="G72" s="1">
+      <c r="G72">
         <v>12</v>
       </c>
-      <c r="H72" s="1">
+      <c r="H72">
         <v>55</v>
       </c>
-      <c r="I72" s="1">
+      <c r="I72">
         <v>0.7</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72">
         <v>4.58</v>
       </c>
     </row>
@@ -2743,28 +2736,28 @@
         <v>2</v>
       </c>
       <c r="C73" t="s">
+        <v>15</v>
+      </c>
+      <c r="D73">
+        <v>0.42033551136363628</v>
+      </c>
+      <c r="E73">
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="F73">
+        <v>3.1</v>
+      </c>
+      <c r="G73">
         <v>16</v>
       </c>
-      <c r="D73">
-        <v>0.2221811931818182</v>
-      </c>
-      <c r="E73">
-        <v>0.94500000000000006</v>
-      </c>
-      <c r="F73">
-        <v>0.78</v>
-      </c>
-      <c r="G73">
-        <v>68</v>
-      </c>
       <c r="H73">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I73">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J73">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
@@ -2775,16 +2768,16 @@
         <v>3</v>
       </c>
       <c r="C74" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D74">
-        <v>0.22237582386363641</v>
+        <v>0.42918119318181819</v>
       </c>
       <c r="E74">
         <v>0.94500000000000006</v>
       </c>
       <c r="F74">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G74">
         <v>68</v>
@@ -2796,7 +2789,7 @@
         <v>0.92</v>
       </c>
       <c r="J74">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
@@ -2807,28 +2800,28 @@
         <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D75">
-        <v>0.22367616477272731</v>
+        <v>0.42937582386363637</v>
       </c>
       <c r="E75">
-        <v>0.49500000000000011</v>
+        <v>0.94500000000000006</v>
       </c>
       <c r="F75">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G75">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H75">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I75">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J75">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
@@ -2842,25 +2835,25 @@
         <v>11</v>
       </c>
       <c r="D76">
-        <v>0.22484394886363629</v>
+        <v>0.43742616477272728</v>
       </c>
       <c r="E76">
-        <v>0.42299999999999999</v>
+        <v>0.49500000000000011</v>
       </c>
       <c r="F76">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G76">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H76">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I76">
         <v>0.95</v>
       </c>
       <c r="J76">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
@@ -2871,10 +2864,10 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D77">
-        <v>0.19447144886363629</v>
+        <v>0.36072144886363627</v>
       </c>
       <c r="E77">
         <v>0.26124999999999998</v>
@@ -2903,28 +2896,28 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
+        <v>15</v>
+      </c>
+      <c r="D78">
+        <v>0.44033551136363641</v>
+      </c>
+      <c r="E78">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="F78">
+        <v>3.1</v>
+      </c>
+      <c r="G78">
         <v>16</v>
       </c>
-      <c r="D78">
-        <v>0.23368119318181821</v>
-      </c>
-      <c r="E78">
-        <v>0.99750000000000005</v>
-      </c>
-      <c r="F78">
-        <v>0.78</v>
-      </c>
-      <c r="G78">
-        <v>68</v>
-      </c>
       <c r="H78">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I78">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J78">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
@@ -2935,16 +2928,16 @@
         <v>3</v>
       </c>
       <c r="C79" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D79">
-        <v>0.2338758238636364</v>
+        <v>0.45218119318181832</v>
       </c>
       <c r="E79">
         <v>0.99750000000000005</v>
       </c>
       <c r="F79">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G79">
         <v>68</v>
@@ -2956,7 +2949,7 @@
         <v>0.92</v>
       </c>
       <c r="J79">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
@@ -2967,28 +2960,28 @@
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D80">
-        <v>0.23555116477272731</v>
+        <v>0.45237582386363639</v>
       </c>
       <c r="E80">
-        <v>0.52250000000000008</v>
+        <v>0.99750000000000005</v>
       </c>
       <c r="F80">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G80">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H80">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I80">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J80">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
@@ -3002,25 +2995,25 @@
         <v>11</v>
       </c>
       <c r="D81">
-        <v>0.2367189488636364</v>
+        <v>0.46117616477272733</v>
       </c>
       <c r="E81">
-        <v>0.44650000000000012</v>
+        <v>0.52250000000000008</v>
       </c>
       <c r="F81">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G81">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H81">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I81">
         <v>0.95</v>
       </c>
       <c r="J81">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
@@ -3031,10 +3024,10 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D82">
-        <v>0.20322144886363641</v>
+        <v>0.37822144886363629</v>
       </c>
       <c r="E82">
         <v>0.27500000000000002</v>
@@ -3063,28 +3056,28 @@
         <v>2</v>
       </c>
       <c r="C83" t="s">
+        <v>15</v>
+      </c>
+      <c r="D83">
+        <v>0.46033551136363632</v>
+      </c>
+      <c r="E83">
+        <v>0.32</v>
+      </c>
+      <c r="F83">
+        <v>3.1</v>
+      </c>
+      <c r="G83">
         <v>16</v>
       </c>
-      <c r="D83">
-        <v>0.24518119318181819</v>
-      </c>
-      <c r="E83">
-        <v>1.05</v>
-      </c>
-      <c r="F83">
-        <v>0.78</v>
-      </c>
-      <c r="G83">
-        <v>68</v>
-      </c>
       <c r="H83">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I83">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J83">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
@@ -3095,16 +3088,16 @@
         <v>3</v>
       </c>
       <c r="C84" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D84">
-        <v>0.24537582386363641</v>
+        <v>0.47518119318181817</v>
       </c>
       <c r="E84">
         <v>1.05</v>
       </c>
       <c r="F84">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G84">
         <v>68</v>
@@ -3116,7 +3109,7 @@
         <v>0.92</v>
       </c>
       <c r="J84">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
@@ -3127,28 +3120,28 @@
         <v>4</v>
       </c>
       <c r="C85" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D85">
-        <v>0.2474261647727273</v>
+        <v>0.47537582386363642</v>
       </c>
       <c r="E85">
-        <v>0.55000000000000004</v>
+        <v>1.05</v>
       </c>
       <c r="F85">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G85">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H85">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I85">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J85">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
@@ -3162,25 +3155,25 @@
         <v>11</v>
       </c>
       <c r="D86">
-        <v>0.24859394886363631</v>
+        <v>0.48492616477272732</v>
       </c>
       <c r="E86">
-        <v>0.47</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F86">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G86">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H86">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I86">
         <v>0.95</v>
       </c>
       <c r="J86">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
@@ -3191,10 +3184,10 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D87">
-        <v>0.21197144886363639</v>
+        <v>0.39572144886363642</v>
       </c>
       <c r="E87">
         <v>0.28875000000000001</v>
@@ -3223,28 +3216,28 @@
         <v>2</v>
       </c>
       <c r="C88" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88">
+        <v>0.48033551136363628</v>
+      </c>
+      <c r="E88">
+        <v>0.33600000000000002</v>
+      </c>
+      <c r="F88">
+        <v>3.1</v>
+      </c>
+      <c r="G88">
         <v>16</v>
       </c>
-      <c r="D88">
-        <v>0.2566811931818182</v>
-      </c>
-      <c r="E88">
-        <v>1.1025</v>
-      </c>
-      <c r="F88">
-        <v>0.78</v>
-      </c>
-      <c r="G88">
-        <v>68</v>
-      </c>
       <c r="H88">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I88">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J88">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
@@ -3255,16 +3248,16 @@
         <v>3</v>
       </c>
       <c r="C89" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D89">
-        <v>0.25687582386363639</v>
+        <v>0.49818119318181819</v>
       </c>
       <c r="E89">
         <v>1.1025</v>
       </c>
       <c r="F89">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G89">
         <v>68</v>
@@ -3276,7 +3269,7 @@
         <v>0.92</v>
       </c>
       <c r="J89">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
@@ -3287,28 +3280,28 @@
         <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D90">
-        <v>0.2593011647727273</v>
+        <v>0.49837582386363638</v>
       </c>
       <c r="E90">
-        <v>0.57750000000000001</v>
+        <v>1.1025</v>
       </c>
       <c r="F90">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G90">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H90">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I90">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J90">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
@@ -3322,25 +3315,25 @@
         <v>11</v>
       </c>
       <c r="D91">
-        <v>0.26046894886363642</v>
+        <v>0.50867616477272726</v>
       </c>
       <c r="E91">
-        <v>0.49349999999999999</v>
+        <v>0.57750000000000001</v>
       </c>
       <c r="F91">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G91">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H91">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I91">
         <v>0.95</v>
       </c>
       <c r="J91">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
@@ -3351,10 +3344,10 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D92">
-        <v>0.2207214488636364</v>
+        <v>0.41322144886363638</v>
       </c>
       <c r="E92">
         <v>0.30249999999999999</v>
@@ -3383,28 +3376,28 @@
         <v>2</v>
       </c>
       <c r="C93" t="s">
+        <v>15</v>
+      </c>
+      <c r="D93">
+        <v>0.50033551136363641</v>
+      </c>
+      <c r="E93">
+        <v>0.35199999999999998</v>
+      </c>
+      <c r="F93">
+        <v>3.1</v>
+      </c>
+      <c r="G93">
         <v>16</v>
       </c>
-      <c r="D93">
-        <v>0.26818119318181821</v>
-      </c>
-      <c r="E93">
-        <v>1.155</v>
-      </c>
-      <c r="F93">
-        <v>0.78</v>
-      </c>
-      <c r="G93">
-        <v>68</v>
-      </c>
       <c r="H93">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I93">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J93">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
@@ -3415,16 +3408,16 @@
         <v>3</v>
       </c>
       <c r="C94" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D94">
-        <v>0.26837582386363629</v>
+        <v>0.52118119318181821</v>
       </c>
       <c r="E94">
         <v>1.155</v>
       </c>
       <c r="F94">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G94">
         <v>68</v>
@@ -3436,7 +3429,7 @@
         <v>0.92</v>
       </c>
       <c r="J94">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
@@ -3447,28 +3440,28 @@
         <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D95">
-        <v>0.27117616477272732</v>
+        <v>0.52137582386363635</v>
       </c>
       <c r="E95">
-        <v>0.60499999999999998</v>
+        <v>1.155</v>
       </c>
       <c r="F95">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G95">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H95">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I95">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J95">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
@@ -3482,25 +3475,25 @@
         <v>11</v>
       </c>
       <c r="D96">
-        <v>0.27234394886363628</v>
+        <v>0.5324261647727272</v>
       </c>
       <c r="E96">
-        <v>0.51700000000000002</v>
+        <v>0.60499999999999998</v>
       </c>
       <c r="F96">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G96">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H96">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I96">
         <v>0.95</v>
       </c>
       <c r="J96">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
@@ -3511,10 +3504,10 @@
         <v>1</v>
       </c>
       <c r="C97" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D97">
-        <v>0.22947144886363641</v>
+        <v>0.43072144886363628</v>
       </c>
       <c r="E97">
         <v>0.31624999999999998</v>
@@ -3543,28 +3536,28 @@
         <v>2</v>
       </c>
       <c r="C98" t="s">
+        <v>15</v>
+      </c>
+      <c r="D98">
+        <v>0.52033551136363632</v>
+      </c>
+      <c r="E98">
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="F98">
+        <v>3.1</v>
+      </c>
+      <c r="G98">
         <v>16</v>
       </c>
-      <c r="D98">
-        <v>0.27968119318181822</v>
-      </c>
-      <c r="E98">
-        <v>1.2075</v>
-      </c>
-      <c r="F98">
-        <v>0.78</v>
-      </c>
-      <c r="G98">
-        <v>68</v>
-      </c>
       <c r="H98">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I98">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J98">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
@@ -3575,16 +3568,16 @@
         <v>3</v>
       </c>
       <c r="C99" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D99">
-        <v>0.27987582386363641</v>
+        <v>0.54418119318181823</v>
       </c>
       <c r="E99">
         <v>1.2075</v>
       </c>
       <c r="F99">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G99">
         <v>68</v>
@@ -3596,7 +3589,7 @@
         <v>0.92</v>
       </c>
       <c r="J99">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
@@ -3607,28 +3600,28 @@
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D100">
-        <v>0.28305116477272729</v>
+        <v>0.54437582386363637</v>
       </c>
       <c r="E100">
-        <v>0.63250000000000006</v>
+        <v>1.2075</v>
       </c>
       <c r="F100">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G100">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H100">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I100">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J100">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
@@ -3642,25 +3635,25 @@
         <v>11</v>
       </c>
       <c r="D101">
-        <v>0.28421894886363641</v>
+        <v>0.55617616477272724</v>
       </c>
       <c r="E101">
-        <v>0.54050000000000009</v>
+        <v>0.63250000000000006</v>
       </c>
       <c r="F101">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G101">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H101">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I101">
         <v>0.95</v>
       </c>
       <c r="J101">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
@@ -3671,10 +3664,10 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D102">
-        <v>0.23822144886363639</v>
+        <v>0.44822144886363641</v>
       </c>
       <c r="E102">
         <v>0.33</v>
@@ -3703,28 +3696,28 @@
         <v>2</v>
       </c>
       <c r="C103" t="s">
+        <v>15</v>
+      </c>
+      <c r="D103">
+        <v>0.54033551136363633</v>
+      </c>
+      <c r="E103">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="F103">
+        <v>3.1</v>
+      </c>
+      <c r="G103">
         <v>16</v>
       </c>
-      <c r="D103">
-        <v>0.29118119318181818</v>
-      </c>
-      <c r="E103">
-        <v>1.26</v>
-      </c>
-      <c r="F103">
-        <v>0.78</v>
-      </c>
-      <c r="G103">
-        <v>68</v>
-      </c>
       <c r="H103">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I103">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J103">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
@@ -3735,16 +3728,16 @@
         <v>3</v>
       </c>
       <c r="C104" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D104">
-        <v>0.29137582386363642</v>
+        <v>0.56718119318181826</v>
       </c>
       <c r="E104">
         <v>1.26</v>
       </c>
       <c r="F104">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G104">
         <v>68</v>
@@ -3756,7 +3749,7 @@
         <v>0.92</v>
       </c>
       <c r="J104">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
@@ -3767,28 +3760,28 @@
         <v>4</v>
       </c>
       <c r="C105" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D105">
-        <v>0.29492616477272732</v>
+        <v>0.56737582386363639</v>
       </c>
       <c r="E105">
-        <v>0.66</v>
+        <v>1.26</v>
       </c>
       <c r="F105">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G105">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H105">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I105">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J105">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
@@ -3802,25 +3795,25 @@
         <v>11</v>
       </c>
       <c r="D106">
-        <v>0.29609394886363632</v>
+        <v>0.57992616477272718</v>
       </c>
       <c r="E106">
-        <v>0.56400000000000006</v>
+        <v>0.66</v>
       </c>
       <c r="F106">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G106">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H106">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I106">
         <v>0.95</v>
       </c>
       <c r="J106">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
@@ -3831,10 +3824,10 @@
         <v>1</v>
       </c>
       <c r="C107" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D107">
-        <v>0.24697144886363639</v>
+        <v>0.46572144886363642</v>
       </c>
       <c r="E107">
         <v>0.34375</v>
@@ -3863,28 +3856,28 @@
         <v>2</v>
       </c>
       <c r="C108" t="s">
+        <v>15</v>
+      </c>
+      <c r="D108">
+        <v>0.56033551136363635</v>
+      </c>
+      <c r="E108">
+        <v>0.4</v>
+      </c>
+      <c r="F108">
+        <v>3.1</v>
+      </c>
+      <c r="G108">
         <v>16</v>
       </c>
-      <c r="D108">
-        <v>0.30268119318181819</v>
-      </c>
-      <c r="E108">
-        <v>1.3125</v>
-      </c>
-      <c r="F108">
-        <v>0.78</v>
-      </c>
-      <c r="G108">
-        <v>68</v>
-      </c>
       <c r="H108">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I108">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J108">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
@@ -3895,16 +3888,16 @@
         <v>3</v>
       </c>
       <c r="C109" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D109">
-        <v>0.30287582386363637</v>
+        <v>0.59018119318181828</v>
       </c>
       <c r="E109">
         <v>1.3125</v>
       </c>
       <c r="F109">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G109">
         <v>68</v>
@@ -3916,7 +3909,7 @@
         <v>0.92</v>
       </c>
       <c r="J109">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
@@ -3927,28 +3920,28 @@
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D110">
-        <v>0.30680116477272729</v>
+        <v>0.59037582386363641</v>
       </c>
       <c r="E110">
-        <v>0.6875</v>
+        <v>1.3125</v>
       </c>
       <c r="F110">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G110">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H110">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I110">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J110">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
@@ -3962,25 +3955,25 @@
         <v>11</v>
       </c>
       <c r="D111">
-        <v>0.30796894886363629</v>
+        <v>0.60367616477272723</v>
       </c>
       <c r="E111">
-        <v>0.58750000000000002</v>
+        <v>0.6875</v>
       </c>
       <c r="F111">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G111">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H111">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I111">
         <v>0.95</v>
       </c>
       <c r="J111">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
@@ -3991,10 +3984,10 @@
         <v>1</v>
       </c>
       <c r="C112" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D112">
-        <v>0.25572144886363629</v>
+        <v>0.48322144886363633</v>
       </c>
       <c r="E112">
         <v>0.35749999999999998</v>
@@ -4023,28 +4016,28 @@
         <v>2</v>
       </c>
       <c r="C113" t="s">
+        <v>15</v>
+      </c>
+      <c r="D113">
+        <v>0.58033551136363637</v>
+      </c>
+      <c r="E113">
+        <v>0.41599999999999998</v>
+      </c>
+      <c r="F113">
+        <v>3.1</v>
+      </c>
+      <c r="G113">
         <v>16</v>
       </c>
-      <c r="D113">
-        <v>0.31418119318181831</v>
-      </c>
-      <c r="E113">
-        <v>1.365</v>
-      </c>
-      <c r="F113">
-        <v>0.78</v>
-      </c>
-      <c r="G113">
-        <v>68</v>
-      </c>
       <c r="H113">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I113">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J113">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
@@ -4055,16 +4048,16 @@
         <v>3</v>
       </c>
       <c r="C114" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D114">
-        <v>0.31437582386363638</v>
+        <v>0.6131811931818183</v>
       </c>
       <c r="E114">
         <v>1.365</v>
       </c>
       <c r="F114">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G114">
         <v>68</v>
@@ -4076,7 +4069,7 @@
         <v>0.92</v>
       </c>
       <c r="J114">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
@@ -4087,28 +4080,28 @@
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D115">
-        <v>0.31867616477272731</v>
+        <v>0.61337582386363643</v>
       </c>
       <c r="E115">
-        <v>0.71500000000000008</v>
+        <v>1.365</v>
       </c>
       <c r="F115">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G115">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H115">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I115">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J115">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
@@ -4122,25 +4115,25 @@
         <v>11</v>
       </c>
       <c r="D116">
-        <v>0.31984394886363637</v>
+        <v>0.62742616477272728</v>
       </c>
       <c r="E116">
-        <v>0.6110000000000001</v>
+        <v>0.71500000000000008</v>
       </c>
       <c r="F116">
-        <v>0.56999999999999995</v>
+        <v>0.51</v>
       </c>
       <c r="G116">
-        <v>32</v>
+        <v>37.5</v>
       </c>
       <c r="H116">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="I116">
         <v>0.95</v>
       </c>
       <c r="J116">
-        <v>2.9375</v>
+        <v>2.9333333333333331</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
@@ -4151,10 +4144,10 @@
         <v>1</v>
       </c>
       <c r="C117" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D117">
-        <v>0.26447144886363633</v>
+        <v>0.50072144886363634</v>
       </c>
       <c r="E117">
         <v>0.37125000000000002</v>
@@ -4183,28 +4176,28 @@
         <v>2</v>
       </c>
       <c r="C118" t="s">
+        <v>15</v>
+      </c>
+      <c r="D118">
+        <v>0.60033551136363628</v>
+      </c>
+      <c r="E118">
+        <v>0.432</v>
+      </c>
+      <c r="F118">
+        <v>3.1</v>
+      </c>
+      <c r="G118">
         <v>16</v>
       </c>
-      <c r="D118">
-        <v>0.32568119318181832</v>
-      </c>
-      <c r="E118">
-        <v>1.4175</v>
-      </c>
-      <c r="F118">
-        <v>0.78</v>
-      </c>
-      <c r="G118">
-        <v>68</v>
-      </c>
       <c r="H118">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I118">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J118">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
@@ -4215,16 +4208,16 @@
         <v>3</v>
       </c>
       <c r="C119" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D119">
-        <v>0.32587582386363639</v>
+        <v>0.63618119318181832</v>
       </c>
       <c r="E119">
         <v>1.4175</v>
       </c>
       <c r="F119">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G119">
         <v>68</v>
@@ -4236,7 +4229,7 @@
         <v>0.92</v>
       </c>
       <c r="J119">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
@@ -4247,28 +4240,28 @@
         <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D120">
-        <v>0.33033551136363631</v>
+        <v>0.63637582386363645</v>
       </c>
       <c r="E120">
-        <v>0.432</v>
+        <v>1.4175</v>
       </c>
       <c r="F120">
-        <v>3.1</v>
+        <v>0.79</v>
       </c>
       <c r="G120">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="H120">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="I120">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="J120">
-        <v>4</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
@@ -4279,10 +4272,10 @@
         <v>5</v>
       </c>
       <c r="C121" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D121">
-        <v>0.33055116477272728</v>
+        <v>0.65117616477272722</v>
       </c>
       <c r="E121">
         <v>0.74250000000000005</v>
@@ -4311,10 +4304,10 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D122">
-        <v>0.27322144886363642</v>
+        <v>0.5182214488636363</v>
       </c>
       <c r="E122">
         <v>0.38500000000000001</v>
@@ -4343,28 +4336,28 @@
         <v>2</v>
       </c>
       <c r="C123" t="s">
+        <v>15</v>
+      </c>
+      <c r="D123">
+        <v>0.62033551136363629</v>
+      </c>
+      <c r="E123">
+        <v>0.44800000000000001</v>
+      </c>
+      <c r="F123">
+        <v>3.1</v>
+      </c>
+      <c r="G123">
         <v>16</v>
       </c>
-      <c r="D123">
-        <v>0.33718119318181822</v>
-      </c>
-      <c r="E123">
-        <v>1.47</v>
-      </c>
-      <c r="F123">
-        <v>0.78</v>
-      </c>
-      <c r="G123">
-        <v>68</v>
-      </c>
       <c r="H123">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I123">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J123">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
@@ -4375,16 +4368,16 @@
         <v>3</v>
       </c>
       <c r="C124" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D124">
-        <v>0.33737582386363629</v>
+        <v>0.65918119318181823</v>
       </c>
       <c r="E124">
         <v>1.47</v>
       </c>
       <c r="F124">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G124">
         <v>68</v>
@@ -4396,7 +4389,7 @@
         <v>0.92</v>
       </c>
       <c r="J124">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
@@ -4407,28 +4400,28 @@
         <v>4</v>
       </c>
       <c r="C125" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D125">
-        <v>0.34033551136363632</v>
+        <v>0.65937582386363636</v>
       </c>
       <c r="E125">
-        <v>0.44800000000000001</v>
+        <v>1.47</v>
       </c>
       <c r="F125">
-        <v>3.1</v>
+        <v>0.79</v>
       </c>
       <c r="G125">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="H125">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="I125">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="J125">
-        <v>4</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
@@ -4439,28 +4432,28 @@
         <v>5</v>
       </c>
       <c r="C126" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D126">
-        <v>0.3424261647727273</v>
+        <v>0.6737045454545455</v>
       </c>
       <c r="E126">
-        <v>0.77</v>
+        <v>0.14699999999999999</v>
       </c>
       <c r="F126">
-        <v>0.51</v>
+        <v>8</v>
       </c>
       <c r="G126">
-        <v>37.5</v>
+        <v>10.65</v>
       </c>
       <c r="H126">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="I126">
-        <v>0.95</v>
+        <v>0.74</v>
       </c>
       <c r="J126">
-        <v>2.9333333333333331</v>
+        <v>1.971830985915493</v>
       </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
@@ -4471,10 +4464,10 @@
         <v>1</v>
       </c>
       <c r="C127" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D127">
-        <v>0.28197144886363629</v>
+        <v>0.53572144886363626</v>
       </c>
       <c r="E127">
         <v>0.39874999999999999</v>
@@ -4503,28 +4496,28 @@
         <v>2</v>
       </c>
       <c r="C128" t="s">
+        <v>15</v>
+      </c>
+      <c r="D128">
+        <v>0.64033551136363631</v>
+      </c>
+      <c r="E128">
+        <v>0.46400000000000002</v>
+      </c>
+      <c r="F128">
+        <v>3.1</v>
+      </c>
+      <c r="G128">
         <v>16</v>
       </c>
-      <c r="D128">
-        <v>0.34868119318181823</v>
-      </c>
-      <c r="E128">
-        <v>1.5225</v>
-      </c>
-      <c r="F128">
-        <v>0.78</v>
-      </c>
-      <c r="G128">
-        <v>68</v>
-      </c>
       <c r="H128">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I128">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J128">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
@@ -4535,16 +4528,16 @@
         <v>3</v>
       </c>
       <c r="C129" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D129">
-        <v>0.34887582386363641</v>
+        <v>0.68218119318181825</v>
       </c>
       <c r="E129">
         <v>1.5225</v>
       </c>
       <c r="F129">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G129">
         <v>68</v>
@@ -4556,7 +4549,7 @@
         <v>0.92</v>
       </c>
       <c r="J129">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
@@ -4567,28 +4560,28 @@
         <v>4</v>
       </c>
       <c r="C130" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D130">
-        <v>0.35033551136363628</v>
+        <v>0.68237582386363638</v>
       </c>
       <c r="E130">
-        <v>0.46400000000000002</v>
+        <v>1.5225</v>
       </c>
       <c r="F130">
-        <v>3.1</v>
+        <v>0.79</v>
       </c>
       <c r="G130">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="H130">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="I130">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="J130">
-        <v>4</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
@@ -4599,28 +4592,28 @@
         <v>5</v>
       </c>
       <c r="C131" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D131">
-        <v>0.35430116477272727</v>
+        <v>0.69220454545454546</v>
       </c>
       <c r="E131">
-        <v>0.79749999999999999</v>
+        <v>0.15225</v>
       </c>
       <c r="F131">
-        <v>0.51</v>
+        <v>8</v>
       </c>
       <c r="G131">
-        <v>37.5</v>
+        <v>10.65</v>
       </c>
       <c r="H131">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="I131">
-        <v>0.95</v>
+        <v>0.74</v>
       </c>
       <c r="J131">
-        <v>2.9333333333333331</v>
+        <v>1.971830985915493</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
@@ -4631,10 +4624,10 @@
         <v>1</v>
       </c>
       <c r="C132" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D132">
-        <v>0.29072144886363638</v>
+        <v>0.55322144886363633</v>
       </c>
       <c r="E132">
         <v>0.41249999999999998</v>
@@ -4663,28 +4656,28 @@
         <v>2</v>
       </c>
       <c r="C133" t="s">
+        <v>15</v>
+      </c>
+      <c r="D133">
+        <v>0.66033551136363633</v>
+      </c>
+      <c r="E133">
+        <v>0.48</v>
+      </c>
+      <c r="F133">
+        <v>3.1</v>
+      </c>
+      <c r="G133">
         <v>16</v>
       </c>
-      <c r="D133">
-        <v>0.36018119318181818</v>
-      </c>
-      <c r="E133">
-        <v>1.575</v>
-      </c>
-      <c r="F133">
-        <v>0.78</v>
-      </c>
-      <c r="G133">
-        <v>68</v>
-      </c>
       <c r="H133">
-        <v>210</v>
+        <v>64</v>
       </c>
       <c r="I133">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J133">
-        <v>3.0882350000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
@@ -4695,28 +4688,28 @@
         <v>3</v>
       </c>
       <c r="C134" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D134">
-        <v>0.36033551136363628</v>
+        <v>0.70518119318181827</v>
       </c>
       <c r="E134">
-        <v>0.48</v>
+        <v>1.575</v>
       </c>
       <c r="F134">
-        <v>3.1</v>
+        <v>0.78</v>
       </c>
       <c r="G134">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="H134">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="I134">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="J134">
-        <v>4</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
@@ -4727,10 +4720,10 @@
         <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D135">
-        <v>0.36037582386363642</v>
+        <v>0.7053758238636364</v>
       </c>
       <c r="E135">
         <v>1.575</v>
@@ -4759,28 +4752,28 @@
         <v>5</v>
       </c>
       <c r="C136" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D136">
-        <v>0.3661761647727273</v>
+        <v>0.71070454545454553</v>
       </c>
       <c r="E136">
-        <v>0.82500000000000007</v>
+        <v>0.1575</v>
       </c>
       <c r="F136">
-        <v>0.51</v>
+        <v>8</v>
       </c>
       <c r="G136">
-        <v>37.5</v>
+        <v>10.65</v>
       </c>
       <c r="H136">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="I136">
-        <v>0.95</v>
+        <v>0.74</v>
       </c>
       <c r="J136">
-        <v>2.9333333333333331</v>
+        <v>1.971830985915493</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
@@ -4791,10 +4784,10 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D137">
-        <v>0.29947144886363641</v>
+        <v>0.57072144886363629</v>
       </c>
       <c r="E137">
         <v>0.42625000000000002</v>
@@ -4823,10 +4816,10 @@
         <v>2</v>
       </c>
       <c r="C138" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D138">
-        <v>0.37033551136363629</v>
+        <v>0.68033551136363635</v>
       </c>
       <c r="E138">
         <v>0.496</v>
@@ -4855,10 +4848,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D139">
-        <v>0.37168119318181819</v>
+        <v>0.72818119318181829</v>
       </c>
       <c r="E139">
         <v>1.6274999999999999</v>
@@ -4887,10 +4880,10 @@
         <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D140">
-        <v>0.37187582386363638</v>
+        <v>0.72837582386363642</v>
       </c>
       <c r="E140">
         <v>1.6274999999999999</v>
@@ -4919,28 +4912,28 @@
         <v>5</v>
       </c>
       <c r="C141" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D141">
-        <v>0.37805116477272732</v>
+        <v>0.72920454545454549</v>
       </c>
       <c r="E141">
-        <v>0.85250000000000004</v>
+        <v>0.16275000000000001</v>
       </c>
       <c r="F141">
-        <v>0.51</v>
+        <v>8</v>
       </c>
       <c r="G141">
-        <v>37.5</v>
+        <v>10.65</v>
       </c>
       <c r="H141">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="I141">
-        <v>0.95</v>
+        <v>0.74</v>
       </c>
       <c r="J141">
-        <v>2.9333333333333331</v>
+        <v>1.971830985915493</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
@@ -4951,10 +4944,10 @@
         <v>1</v>
       </c>
       <c r="C142" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D142">
-        <v>0.30822144886363628</v>
+        <v>0.58822144886363625</v>
       </c>
       <c r="E142">
         <v>0.44</v>
@@ -4983,10 +4976,10 @@
         <v>2</v>
       </c>
       <c r="C143" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D143">
-        <v>0.38033551136363641</v>
+        <v>0.70033551136363636</v>
       </c>
       <c r="E143">
         <v>0.51200000000000001</v>
@@ -5018,25 +5011,25 @@
         <v>16</v>
       </c>
       <c r="D144">
-        <v>0.38318119318181831</v>
+        <v>0.74770454545454546</v>
       </c>
       <c r="E144">
-        <v>1.68</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="F144">
-        <v>0.78</v>
+        <v>8</v>
       </c>
       <c r="G144">
-        <v>68</v>
+        <v>10.65</v>
       </c>
       <c r="H144">
-        <v>210</v>
+        <v>21</v>
       </c>
       <c r="I144">
-        <v>0.92</v>
+        <v>0.74</v>
       </c>
       <c r="J144">
-        <v>3.0882350000000001</v>
+        <v>1.971830985915493</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
@@ -5047,16 +5040,16 @@
         <v>4</v>
       </c>
       <c r="C145" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D145">
-        <v>0.38337582386363639</v>
+        <v>0.75118119318181831</v>
       </c>
       <c r="E145">
         <v>1.68</v>
       </c>
       <c r="F145">
-        <v>0.79</v>
+        <v>0.78</v>
       </c>
       <c r="G145">
         <v>68</v>
@@ -5068,7 +5061,7 @@
         <v>0.92</v>
       </c>
       <c r="J145">
-        <v>3.0882352941176472</v>
+        <v>3.0882350000000001</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.35">
@@ -5079,28 +5072,28 @@
         <v>5</v>
       </c>
       <c r="C146" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D146">
-        <v>0.38992616477272729</v>
+        <v>0.75137582386363644</v>
       </c>
       <c r="E146">
-        <v>0.88</v>
+        <v>1.68</v>
       </c>
       <c r="F146">
-        <v>0.51</v>
+        <v>0.79</v>
       </c>
       <c r="G146">
-        <v>37.5</v>
+        <v>68</v>
       </c>
       <c r="H146">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="I146">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="J146">
-        <v>2.9333333333333331</v>
+        <v>3.0882352941176472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>